<commit_message>
fix: add new protein
</commit_message>
<xml_diff>
--- a/protein without pdb files of high quality-need itasser.xlsx
+++ b/protein without pdb files of high quality-need itasser.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luho/Documents/GitHub/De-nevo-protein-3D-structure-yeast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A40C821-446A-CD45-8595-A58D8B43C511}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4CA3752-6B29-CE4E-A9E2-C1F67EF07143}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7340" yWindow="5240" windowWidth="27780" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6180" yWindow="2380" windowWidth="27780" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="protein without pdb files of hi" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" concurrentCalc="0"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -2955,7 +2955,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3153,8 +3153,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -3269,6 +3275,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -3314,11 +3335,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3679,7 +3702,7 @@
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="36.1640625" customWidth="1"/>
+    <col min="3" max="3" width="39.5" customWidth="1"/>
     <col min="4" max="4" width="24.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3768,7 +3791,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B7" t="s">
@@ -3782,7 +3805,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B8" t="s">
@@ -3796,7 +3819,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="A9" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B9" t="s">
@@ -4230,7 +4253,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="A40" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B40" t="s">
@@ -4244,7 +4267,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+      <c r="A41" s="5" t="s">
         <v>61</v>
       </c>
       <c r="B41" t="s">
@@ -4258,7 +4281,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+      <c r="A42" s="5" t="s">
         <v>62</v>
       </c>
       <c r="B42" t="s">
@@ -4272,7 +4295,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+      <c r="A43" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B43" t="s">
@@ -4286,7 +4309,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+      <c r="A44" s="5" t="s">
         <v>63</v>
       </c>
       <c r="B44" t="s">
@@ -4300,7 +4323,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+      <c r="A45" s="5" t="s">
         <v>64</v>
       </c>
       <c r="B45" t="s">
@@ -4314,7 +4337,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+      <c r="A46" s="5" t="s">
         <v>65</v>
       </c>
       <c r="B46" t="s">
@@ -4328,7 +4351,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+      <c r="A47" s="5" t="s">
         <v>66</v>
       </c>
       <c r="B47" t="s">
@@ -20261,5 +20284,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add a new protein
</commit_message>
<xml_diff>
--- a/protein without pdb files of high quality-need itasser.xlsx
+++ b/protein without pdb files of high quality-need itasser.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luho/Documents/GitHub/De-nevo-protein-3D-structure-yeast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4CA3752-6B29-CE4E-A9E2-C1F67EF07143}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B808192-52DC-FA4F-9E1B-A73017611861}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6180" yWindow="2380" windowWidth="27780" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14040" yWindow="10560" windowWidth="27780" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="protein without pdb files of hi" sheetId="1" r:id="rId1"/>
@@ -3149,13 +3149,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
+        <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3340,8 +3340,8 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3791,7 +3791,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B7" t="s">
@@ -3819,7 +3819,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="5" t="s">
         <v>18</v>
       </c>
       <c r="B9" t="s">
@@ -3833,7 +3833,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="A10" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B10" t="s">
@@ -4253,7 +4253,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="4" t="s">
         <v>58</v>
       </c>
       <c r="B40" t="s">
@@ -4267,7 +4267,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="4" t="s">
         <v>61</v>
       </c>
       <c r="B41" t="s">
@@ -4281,7 +4281,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="4" t="s">
         <v>62</v>
       </c>
       <c r="B42" t="s">
@@ -4295,7 +4295,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B43" t="s">
@@ -4309,7 +4309,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="4" t="s">
         <v>63</v>
       </c>
       <c r="B44" t="s">
@@ -4323,7 +4323,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="5" t="s">
+      <c r="A45" s="4" t="s">
         <v>64</v>
       </c>
       <c r="B45" t="s">
@@ -4337,7 +4337,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B46" t="s">
@@ -4351,7 +4351,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="5" t="s">
+      <c r="A47" s="4" t="s">
         <v>66</v>
       </c>
       <c r="B47" t="s">

</xml_diff>

<commit_message>
feat: add new protein
</commit_message>
<xml_diff>
--- a/protein without pdb files of high quality-need itasser.xlsx
+++ b/protein without pdb files of high quality-need itasser.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luho/Documents/GitHub/De-nevo-protein-3D-structure-yeast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B808192-52DC-FA4F-9E1B-A73017611861}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2E2138-0BEC-034B-BE6E-5C672DA5F27F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14040" yWindow="10560" windowWidth="27780" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9700" yWindow="4060" windowWidth="27780" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="protein without pdb files of hi" sheetId="1" r:id="rId1"/>
@@ -2819,7 +2819,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2950,6 +2950,13 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0" tint="-0.499984740745262"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3155,7 +3162,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3337,11 +3344,11 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3700,7 +3707,7 @@
   <dimension ref="A1:D1184"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="39.5" customWidth="1"/>
     <col min="4" max="4" width="24.33203125" customWidth="1"/>
@@ -3721,7 +3728,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
@@ -3735,7 +3742,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
@@ -3749,7 +3756,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B4" t="s">
@@ -3763,7 +3770,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B5" t="s">
@@ -3777,7 +3784,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B6" t="s">
@@ -3791,7 +3798,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B7" t="s">
@@ -3805,7 +3812,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B8" t="s">
@@ -3847,7 +3854,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
@@ -4253,7 +4260,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B40" t="s">
@@ -4267,7 +4274,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B41" t="s">
@@ -4281,7 +4288,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B42" t="s">
@@ -4295,7 +4302,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B43" t="s">
@@ -4309,7 +4316,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B44" t="s">
@@ -4323,7 +4330,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="4" t="s">
+      <c r="A45" s="1" t="s">
         <v>64</v>
       </c>
       <c r="B45" t="s">
@@ -4337,7 +4344,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B46" t="s">
@@ -4351,7 +4358,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B47" t="s">

</xml_diff>

<commit_message>
feat: add new potein structure
</commit_message>
<xml_diff>
--- a/protein without pdb files of high quality-need itasser.xlsx
+++ b/protein without pdb files of high quality-need itasser.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luho/Documents/GitHub/De-nevo-protein-3D-structure-yeast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5C5214-860A-454B-A1D7-D03F385C36C1}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B758D19-7FFF-FA4D-AC84-D8A15121D89F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9580" yWindow="4060" windowWidth="27780" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="220" yWindow="460" windowWidth="27780" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="protein without pdb files of hi" sheetId="1" r:id="rId1"/>
@@ -2962,7 +2962,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3172,6 +3172,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -3348,7 +3354,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3356,6 +3362,7 @@
     <xf numFmtId="0" fontId="18" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="37" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4267,7 +4274,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="7" t="s">
         <v>58</v>
       </c>
       <c r="B40" t="s">
@@ -4281,7 +4288,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
+      <c r="A41" s="7" t="s">
         <v>61</v>
       </c>
       <c r="B41" t="s">
@@ -4295,7 +4302,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="6" t="s">
         <v>62</v>
       </c>
       <c r="B42" t="s">

</xml_diff>